<commit_message>
Database document excel updated 21-08
</commit_message>
<xml_diff>
--- a/Documents/Database.xlsx
+++ b/Documents/Database.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ZensarDemos\Capstone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ZensarDemos\Capstone\repo\BankingApp\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80108DDF-EF13-4D47-B5EC-C85F5979E269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37475D4-AE8E-488E-A703-778984378DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{149B8D31-B82A-4DB2-BA4C-3A3A58D8C5B0}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="71">
   <si>
     <t>CREATE TABLE Users (</t>
   </si>
@@ -156,6 +156,102 @@
   </si>
   <si>
     <t>New, Active, Closed</t>
+  </si>
+  <si>
+    <t>CREATE TABLE LoanApplication (</t>
+  </si>
+  <si>
+    <t>ApplicationId INT IDENTITY(1,1) PRIMARY KEY,</t>
+  </si>
+  <si>
+    <t>CustomerId INT NOT NULL,</t>
+  </si>
+  <si>
+    <t>LoanTenureMonths INT NOT NULL,</t>
+  </si>
+  <si>
+    <t>AnnualIncome DECIMAL(18,2) NOT NULL,</t>
+  </si>
+  <si>
+    <t>ApplicationDate DATETIME NOT NULL DEFAULT GETDATE(),</t>
+  </si>
+  <si>
+    <t>Status VARCHAR(20) NOT NULL DEFAULT 'Submitted',</t>
+  </si>
+  <si>
+    <t>CONSTRAINT FK_LoanApplication_Customers</t>
+  </si>
+  <si>
+    <t>FOREIGN KEY (CustomerId)</t>
+  </si>
+  <si>
+    <t>REFERENCES Customers(CustomerId)</t>
+  </si>
+  <si>
+    <t>ApplicationId INT NOT NULL,</t>
+  </si>
+  <si>
+    <t>CONSTRAINT FK_Loans_LoanApplication</t>
+  </si>
+  <si>
+    <t>FOREIGN KEY (ApplicationId)</t>
+  </si>
+  <si>
+    <t>REFERENCES LoanApplication(ApplicationId)</t>
+  </si>
+  <si>
+    <t>CREATE TABLE CreditAssessment (</t>
+  </si>
+  <si>
+    <t>AssessmentId INT IDENTITY(1,1) PRIMARY KEY,</t>
+  </si>
+  <si>
+    <t>IsValid BIT NOT NULL,</t>
+  </si>
+  <si>
+    <t>IsEligible BIT NOT NULL,</t>
+  </si>
+  <si>
+    <t>RiskScore INT NOT NULL,</t>
+  </si>
+  <si>
+    <t>Decision VARCHAR(20) NOT NULL,</t>
+  </si>
+  <si>
+    <t>AssessmentDate DATETIME NOT NULL DEFAULT GETDATE(),</t>
+  </si>
+  <si>
+    <t>CONSTRAINT FK_CreditAssessment_LoanApplication</t>
+  </si>
+  <si>
+    <t>Approved, Rejected</t>
+  </si>
+  <si>
+    <t>ApplicationId | CustomerId | LoanAmount | Tenure | AnnualIncome | Status</t>
+  </si>
+  <si>
+    <t>------------- | ---------- | ---------- | ------- | ------------ | ----------</t>
+  </si>
+  <si>
+    <t>1 | 1 | 500000 | 60 | 1200000 | Approved</t>
+  </si>
+  <si>
+    <t>2 | 2 | 2000000 | 120 | 600000 | Rejected</t>
+  </si>
+  <si>
+    <t>AssessmentId | ApplicationId | IsValid | IsEligible | RiskScore | Decision</t>
+  </si>
+  <si>
+    <t>------------ | ------------- | ------- | ---------- | --------- | ------------</t>
+  </si>
+  <si>
+    <t>1 | 1 | 1 | 1 | 85 | Approved</t>
+  </si>
+  <si>
+    <t>2 | 2 | 1 | 0 | 45 | Rejected</t>
+  </si>
+  <si>
+    <t>Submitted,Approved,Rejected</t>
   </si>
 </sst>
 </file>
@@ -536,11 +632,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65BF9D2D-18E2-4264-955E-478FAD00F1D7}">
-  <dimension ref="B2:M52"/>
+  <dimension ref="B2:M88"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="59.08984375" customWidth="1"/>
     <col min="3" max="3" width="46.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="62.6328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.7265625" customWidth="1"/>
     <col min="13" max="13" width="57.453125" customWidth="1"/>
   </cols>
@@ -746,23 +843,193 @@
         <v>31</v>
       </c>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B48" t="s">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B47" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B49" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B49" t="s">
+    <row r="50" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B50" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B50" t="s">
+    <row r="51" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B51" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B52" t="s">
+    <row r="53" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="54" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B54" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="55" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B55" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B56" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B59" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="60" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B60" t="s">
+        <v>40</v>
+      </c>
+      <c r="D60" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="61" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B61" t="s">
+        <v>41</v>
+      </c>
+      <c r="D61" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="62" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B62" t="s">
+        <v>28</v>
+      </c>
+      <c r="D62" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="63" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B63" t="s">
+        <v>42</v>
+      </c>
+      <c r="D63" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="64" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B64" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="65" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B65" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="66" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B66" t="s">
+        <v>45</v>
+      </c>
+      <c r="C66" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="68" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B68" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="69" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B69" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="70" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B70" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="71" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B71" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B75" t="s">
+        <v>53</v>
+      </c>
+      <c r="D75" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="76" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B76" t="s">
+        <v>54</v>
+      </c>
+      <c r="D76" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="77" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B77" t="s">
+        <v>49</v>
+      </c>
+      <c r="D77" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="78" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B78" t="s">
+        <v>55</v>
+      </c>
+      <c r="D78" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="79" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B79" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="80" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B80" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="81" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B81" t="s">
+        <v>58</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="82" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B82" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="84" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B84" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="85" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B85" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="86" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B86" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="88" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B88" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>